<commit_message>
Finalize QA'd backlink audit, disavow and baseline Excel deliverables
Merge 3 QA-agent reviews of borderline domains into final verdicts and
regenerate workbooks.

Final classification (1,170 referring domains / 3,651 backlinks reviewed):
- TOXIC   1,057 (90.3%) -> disavow candidates
- KEEP      103
- MONITOR     5
- OWN         5 (client/sister properties, never disavowed)

Deliverables:
- MasterLawn_Backlink_Audit.xlsx (per-domain + per-backlink classification,
  anchors, distributions, toxic-IP clusters, methodology)
- MasterLawn_Disavow.xlsx + disavow_masterlawn.txt (1,057 domain-level entries)
- MasterLawn_Baseline_Benchmark.xlsx (critical Semrush baseline)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EcadPGkZjcYFPLYRDHxo
</commit_message>
<xml_diff>
--- a/seo/MasterLawn_Baseline_Benchmark.xlsx
+++ b/seo/MasterLawn_Baseline_Benchmark.xlsx
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>887</v>
+        <v>1057</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>75.8%</t>
+          <t>90.3%</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1049,7 +1049,7 @@
         <v>1167</v>
       </c>
       <c r="D3" t="n">
-        <v>887</v>
+        <v>1057</v>
       </c>
       <c r="E3" t="n">
         <v>2525</v>

</xml_diff>

<commit_message>
Consolidate two-pass QA into final deliverables + add index/notes
Final classification after critical adversarial second pass:
- TOXIC   1,003 (85.7%)  -> disavow candidates
- KEEP      113
- MONITOR    49
- OWN         5

Regenerate all three workbooks with qa2 overrides; add README_DELIVERABLES.md
documenting every file/sheet, the QA method, and formatting.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EcadPGkZjcYFPLYRDHxo
</commit_message>
<xml_diff>
--- a/seo/MasterLawn_Baseline_Benchmark.xlsx
+++ b/seo/MasterLawn_Baseline_Benchmark.xlsx
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1057</v>
+        <v>1003</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>90.3%</t>
+          <t>85.7%</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1049,7 +1049,7 @@
         <v>1167</v>
       </c>
       <c r="D3" t="n">
-        <v>1057</v>
+        <v>1003</v>
       </c>
       <c r="E3" t="n">
         <v>2525</v>

</xml_diff>

<commit_message>
Upgrade standalone Disavow + Baseline workbooks to match audit design
- MasterLawn_Disavow.xlsx: banner, numbered zebra table with reason, README
- MasterLawn_Baseline_Benchmark.xlsx: KPI tiles + sectioned Semrush metrics,
  local keyword set, change log
- refresh disavow_masterlawn.txt (1,003 domains)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EcadPGkZjcYFPLYRDHxo
</commit_message>
<xml_diff>
--- a/seo/MasterLawn_Baseline_Benchmark.xlsx
+++ b/seo/MasterLawn_Baseline_Benchmark.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,25 +28,71 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="16"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="0052514E"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="0052514E"/>
+      <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000D366B"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00E34948"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000D366B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000B0B0B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000D366B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0052514E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -55,12 +101,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="000D366B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="00E8F0FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00184F95"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,29 +135,50 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9DEE6"/>
       </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9DEE6"/>
       </right>
       <top style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9DEE6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9DEE6"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -464,403 +546,523 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="B2:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Master Lawn — Critical SEO Baseline Benchmark</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Source: Semrush  |  Snapshot date: 2026-09-04  |  Frozen 'before' state for measuring disavow + rebuild impact</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>MASTER LAWN — CRITICAL SEO BASELINE BENCHMARK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Source: Semrush (Authority Score &amp; Traffic)  ·  Snapshot 2026-09-04  ·  Frozen 'before' state for measuring disavow + rebuild impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>AUTHORITY SCORE</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>REFERRING DOMAINS</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL BACKLINKS</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>% TOXIC</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="7" t="n">
+        <v>1167</v>
+      </c>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="7" t="n">
+        <v>3613</v>
+      </c>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>85.7%</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>ORGANIC KEYWORDS</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>ORGANIC TRAFFIC / MO</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>TRAFFIC VALUE / MO</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>TOXIC DOMAINS</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="n">
+        <v>2525</v>
+      </c>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="7" t="n">
+        <v>2391</v>
+      </c>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>$10,324</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="8" t="n">
+        <v>1003</v>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>AUTHORITY &amp; BACKLINK PROFILE (Semrush)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    </row>
+    <row r="14">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Authority Score</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C14" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Low; inflated by spam volume, not earned trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>inflated by spam volume, not earned trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Total backlinks</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="C15" s="11" t="n">
         <v>3613</v>
       </c>
-      <c r="C6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Referring domains</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="C16" s="11" t="n">
         <v>1167</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>≈90% at Authority Score &lt;=6 (spam/PBN bulk)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Referring IPs</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1151</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>~90% at Authority Score ≤6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Referring IPs (Class C)</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>792</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Follow backlinks</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>2877</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Nofollow backlinks</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>743</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Sponsored / UGC</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>0 / 5</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>1,151 (792)</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Follow / Nofollow</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>2,877 / 743</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Text / Image links</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>3243 / 104</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>TOXICITY (this audit)</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Referring domains classified TOXIC</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>3,243 / 104</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>TOXICITY (this audit, 2 QA passes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>TOXIC — disavow</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
         <v>1003</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>recommend disavow</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Referring domains MONITOR</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>85.7% of referring domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>113</v>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>legitimate / relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
         <v>49</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>human QA</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Referring domains KEEP</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>113</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>legitimate/relevant</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Referring domains OWN</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>watch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>OWN</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>client/sister properties</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>% toxic</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>85.7%</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>client / sister properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Recency</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>~94% first seen 2026</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>active negative-SEO blast</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>ORGANIC VISIBILITY (Semrush, US)</t>
         </is>
       </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    </row>
+    <row r="29">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Semrush Rank</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="C29" s="11" t="n">
         <v>595080</v>
       </c>
-      <c r="C23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Organic keywords</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="C30" s="11" t="n">
         <v>2525</v>
       </c>
-      <c r="C24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Keywords in positions 1-3</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>104</v>
-      </c>
-      <c r="C25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Keywords in positions 4-10</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>235</v>
-      </c>
-      <c r="C26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Keywords in positions 11-20</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>223</v>
-      </c>
-      <c r="C27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Organic traffic / month</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>104 in top 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Organic traffic / mo</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n">
         <v>2391</v>
       </c>
-      <c r="C28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Organic traffic value / month (USD)</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>10324</v>
-      </c>
-      <c r="C29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Organic traffic value / mo</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>$10,324</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Paid keywords / traffic</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>0 / 0</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>PENDING CLIENT ACCESS (source of truth once granted)</t>
         </is>
       </c>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    </row>
+    <row r="36">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Google Search Console</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>clicks / impressions / CTR / avg position</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>clicks / impressions / CTR / position</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>request access</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>GA4</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>organic sessions &amp; conversions</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>request access</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Rank tracker (local pack)</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Semrush Position Tracking</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
         <is>
           <t>to configure</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Memphis/Germantown/Bartlett/Olive Branch/Huntsville</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    </row>
+    <row r="39">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Confirm ownership</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>masterlawninc.com / masterlawn.org / .net / midsouthturf / greenkingspray</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>masterlawninc / .org / .net / midsouthturf / greenkingspray</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="62">
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B6:C7"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="E39:I39"/>
+    <mergeCell ref="E14:I14"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="E19:I19"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="D10:E11"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E15:I15"/>
+    <mergeCell ref="F10:G11"/>
+    <mergeCell ref="H10:I11"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="D6:E7"/>
+    <mergeCell ref="F6:G7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="H6:I7"/>
+    <mergeCell ref="E16:I16"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="E18:I18"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -874,23 +1076,29 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="88" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>LOCAL KEYWORD SET</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Geo modifiers to track</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -976,6 +1184,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -992,50 +1203,56 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>CHANGE LOG (add a row monthly)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Authority Score</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Ref domains</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Toxic domains</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Toxic</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>Organic KW</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Organic traffic/mo</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Traffic/mo</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1064,6 +1281,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add local-citation safeguard + dedupe referring domains
Address risk of disavowing genuine local-business directory citations:
- link-level analysis: 844 toxic domains use real city/service anchors, but 806
  are camouflage (on PBN farms/throwaway hosts); 16 standalone local directories
  moved TOXIC->MONITOR (excluded from disavow)
- new "Local Citations Review" sheet lists every geo-anchor link with on-farm flag,
  example anchor + target page, and default recommendation for human review
- dedupe referring domains by root (Semrush returned topleveldomains.space twice)

Final: 1,169 unique referring domains -> TOXIC 986 | KEEP 113 | MONITOR 65 | OWN 5.
Disavow = 986 (txt = sheet = unique). All workbooks + markdown updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EcadPGkZjcYFPLYRDHxo
</commit_message>
<xml_diff>
--- a/seo/MasterLawn_Baseline_Benchmark.xlsx
+++ b/seo/MasterLawn_Baseline_Benchmark.xlsx
@@ -615,7 +615,7 @@
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>84.3%</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -672,7 +672,7 @@
       </c>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="8" t="n">
-        <v>1003</v>
+        <v>986</v>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
@@ -787,11 +787,11 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>1003</v>
+        <v>986</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>85.7% of referring domains</t>
+          <t>84.3% of referring domains</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
         <v>1167</v>
       </c>
       <c r="D3" t="n">
-        <v>1003</v>
+        <v>986</v>
       </c>
       <c r="E3" t="n">
         <v>2525</v>

</xml_diff>

<commit_message>
Apply nofollow policy: disavow only dofollow spam
Nofollow links pass no PageRank, so all-nofollow toxic domains carry ~no
algorithmic risk and are kept out of the disavow (low-quality nofollow directory
listings can aid GMB/local NAP). Only dofollow spam + clearly malicious verticals
(e.g. truebookies.com gambling) stay disavowed.

- 70 all-nofollow non-malicious toxic domains moved TOXIC->MONITOR
- add Dofollow/Nofollow per-domain columns to Referring Domains sheet
- methodology + README + baseline document the policy

Final: 1,169 unique referring domains -> TOXIC 916 | KEEP 113 | MONITOR 135 | OWN 5.
Disavow = 916 (txt = sheet).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EcadPGkZjcYFPLYRDHxo
</commit_message>
<xml_diff>
--- a/seo/MasterLawn_Baseline_Benchmark.xlsx
+++ b/seo/MasterLawn_Baseline_Benchmark.xlsx
@@ -615,7 +615,7 @@
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>84.3%</t>
+          <t>78.4%</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -672,7 +672,7 @@
       </c>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="8" t="n">
-        <v>986</v>
+        <v>916</v>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
@@ -787,11 +787,11 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>986</v>
+        <v>916</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>84.3% of referring domains</t>
+          <t>78.4% of referring domains</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>65</v>
+        <v>135</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
         <v>1167</v>
       </c>
       <c r="D3" t="n">
-        <v>986</v>
+        <v>916</v>
       </c>
       <c r="E3" t="n">
         <v>2525</v>

</xml_diff>

<commit_message>
Add organic-traffic proof; spare low-traffic domains from disavow
Verify "are these real directories?" via organic traffic (Ahrefs): a functioning
citation directory that aids GMB is indexed and gets traffic; a dead PBN page has
zero. Findings:
- every real citation directory with traffic (yellowpages, bbb, birdeye, superpages,
  dexknows, citysquares, neustarlocaleze, chambers, agreatertown...) is already KEPT
- 852 of the 865 disavow domains have EXACTLY zero organic traffic
- the 13 with a negligible trickle (1-28/mo) moved TOXIC->MONITOR (held for review)
- add "Org traffic" column to Referring Domains + Disavow sheets

Final: TOXIC 852 (all zero-traffic + hard evidence) | KEEP 113 | MONITOR 199 | OWN 5.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EcadPGkZjcYFPLYRDHxo
</commit_message>
<xml_diff>
--- a/seo/MasterLawn_Baseline_Benchmark.xlsx
+++ b/seo/MasterLawn_Baseline_Benchmark.xlsx
@@ -615,7 +615,7 @@
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>72.9%</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -672,7 +672,7 @@
       </c>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="8" t="n">
-        <v>865</v>
+        <v>852</v>
       </c>
       <c r="I10" s="6" t="n"/>
     </row>
@@ -787,11 +787,11 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>865</v>
+        <v>852</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>74.0% of referring domains</t>
+          <t>72.9% of referring domains</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
         <v>1167</v>
       </c>
       <c r="D3" t="n">
-        <v>865</v>
+        <v>852</v>
       </c>
       <c r="E3" t="n">
         <v>2525</v>

</xml_diff>